<commit_message>
testing out the sheet
</commit_message>
<xml_diff>
--- a/lcoe_plots/bio_ethylene_lcoe/LCOE_BIO_Ethylene.xlsx
+++ b/lcoe_plots/bio_ethylene_lcoe/LCOE_BIO_Ethylene.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abbie/MacroEnergy-Abbie.jl/MacroEnergyExamples/lcoe_plots/bio_ethylene_lcoe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8908703-CD10-134A-91B7-D5C39B013544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B827847F-8785-4648-8AC3-7EECB8A4E5C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lc_detailed" sheetId="1" r:id="rId1"/>
@@ -1078,8 +1078,8 @@
     <col min="124" max="124" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="125" max="125" width="26.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="126" max="126" width="21.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="127" max="135" width="10.83203125" style="1" customWidth="1"/>
-    <col min="136" max="16384" width="10.83203125" style="1"/>
+    <col min="127" max="136" width="10.83203125" style="1" customWidth="1"/>
+    <col min="137" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:126" x14ac:dyDescent="0.2">
@@ -8867,772 +8867,772 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B1:Y58"/>
+  <dimension ref="A1:X58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="42.5" style="22" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" style="22" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" style="22" customWidth="1"/>
-    <col min="5" max="5" width="14.5" style="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" style="22" customWidth="1"/>
-    <col min="7" max="7" width="18.1640625" style="22" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" style="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.1640625" style="22" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" style="22" customWidth="1"/>
-    <col min="11" max="11" width="12.5" style="22" customWidth="1"/>
-    <col min="12" max="12" width="8.5" style="22" customWidth="1"/>
-    <col min="13" max="13" width="11.33203125" style="22" customWidth="1"/>
-    <col min="14" max="14" width="10.5" style="22" customWidth="1"/>
-    <col min="15" max="15" width="15.33203125" style="22" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" style="22" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" style="22" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.6640625" style="22" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.6640625" style="22" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.83203125" style="22" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.6640625" style="22" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="3.5" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.5" style="22" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" style="22" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="22" customWidth="1"/>
+    <col min="4" max="4" width="14.5" style="22" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1640625" style="22" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" style="22" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" style="22" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" style="22" customWidth="1"/>
+    <col min="10" max="10" width="12.5" style="22" customWidth="1"/>
+    <col min="11" max="11" width="8.5" style="22" customWidth="1"/>
+    <col min="12" max="12" width="11.33203125" style="22" customWidth="1"/>
+    <col min="13" max="13" width="10.5" style="22" customWidth="1"/>
+    <col min="14" max="14" width="15.33203125" style="22" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" style="22" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" style="22" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.83203125" style="22" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.5" customWidth="1"/>
+    <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B1" s="21" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="W1" s="28" t="s">
+      <c r="V1" s="28" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="23" t="s">
+        <v>68</v>
+      </c>
       <c r="B2" s="23" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="O2" s="23" t="s">
         <v>84</v>
       </c>
+      <c r="O2" s="24" t="s">
+        <v>86</v>
+      </c>
       <c r="P2" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q2" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="R2" s="24" t="s">
         <v>85</v>
       </c>
+      <c r="R2" s="25" t="s">
+        <v>70</v>
+      </c>
       <c r="S2" s="25" t="s">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="T2" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="U2" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="W2" t="s">
+      <c r="V2" t="s">
         <v>126</v>
       </c>
-      <c r="X2">
+      <c r="W2">
         <v>45.6</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="X2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="30" t="str">
+    <row r="3" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="30" t="str">
         <f>lc_detailed!AZ3</f>
         <v>SE_Ethanol_Dehydration_NGfuel</v>
       </c>
+      <c r="B3" s="31">
+        <f>lc_detailed!BH3/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C3" s="31">
-        <f>lc_detailed!BH3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI3/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D3" s="31">
-        <f>lc_detailed!BI3/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ3/$W$2</f>
+        <v>0.15214611962784025</v>
       </c>
       <c r="E3" s="31">
-        <f>lc_detailed!BJ3/$X$2</f>
-        <v>0.15214611962784025</v>
+        <f>lc_detailed!BK3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F3" s="31">
-        <f>lc_detailed!BK3/$X$2</f>
+        <f>lc_detailed!BL3/$W$2</f>
         <v>0</v>
       </c>
       <c r="G3" s="31">
-        <f>lc_detailed!BL3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BM3/$W$2</f>
+        <v>0.16956915850640997</v>
       </c>
       <c r="H3" s="31">
-        <f>lc_detailed!BM3/$X$2</f>
-        <v>0.16956915850640997</v>
+        <f>lc_detailed!BN3/$W$2</f>
+        <v>0.34050656770373977</v>
       </c>
       <c r="I3" s="31">
-        <f>lc_detailed!BN3/$X$2</f>
-        <v>0.34050656770373977</v>
+        <f>lc_detailed!BO3/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J3" s="31">
-        <f>lc_detailed!BO3/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K3" s="31">
-        <f>lc_detailed!BP3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ3/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L3" s="31">
-        <f>lc_detailed!BQ3/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR3/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M3" s="31">
-        <f>lc_detailed!BR3/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS3/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N3" s="31">
-        <f>lc_detailed!BS3/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT3/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O3" s="31">
-        <f>lc_detailed!BT3/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!CB3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P3" s="31">
-        <f>lc_detailed!CB3/$X$2</f>
+        <f>lc_detailed!CC3/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q3" s="31">
-        <f>lc_detailed!CC3/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R3" s="31">
         <f>lc_detailed!CA3</f>
         <v>0</v>
       </c>
-      <c r="S3" s="32">
+      <c r="R3" s="32">
         <f>lc_detailed!BE3</f>
         <v>493.01210108179316</v>
       </c>
+      <c r="S3" s="32">
+        <f t="shared" ref="S3:S10" si="0">R3/$W$2</f>
+        <v>10.811668883372656</v>
+      </c>
       <c r="T3" s="32">
-        <f t="shared" ref="T3:T10" si="0">S3/$X$2</f>
-        <v>10.811668883372656</v>
-      </c>
-      <c r="U3" s="32">
-        <f t="shared" ref="U3:U10" si="1">SUM(C3:Q3)</f>
+        <f t="shared" ref="T3:T10" si="1">SUM(B3:P3)</f>
         <v>10.811668883372658</v>
       </c>
     </row>
-    <row r="4" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="30" t="str">
+    <row r="4" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="30" t="str">
         <f>lc_detailed!AZ4</f>
         <v>SE_Ethanol_Dehydration_H2fuel</v>
       </c>
+      <c r="B4" s="31">
+        <f>lc_detailed!BH4/$W$2</f>
+        <v>0.30171339336527736</v>
+      </c>
       <c r="C4" s="31">
-        <f>lc_detailed!BH4/$X$2</f>
-        <v>0.30171339336527736</v>
+        <f>lc_detailed!BI4/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D4" s="31">
-        <f>lc_detailed!BI4/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ4/$W$2</f>
+        <v>0.15214611962784025</v>
       </c>
       <c r="E4" s="31">
-        <f>lc_detailed!BJ4/$X$2</f>
-        <v>0.15214611962784025</v>
+        <f>lc_detailed!BK4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F4" s="31">
-        <f>lc_detailed!BK4/$X$2</f>
+        <f>lc_detailed!BL4/$W$2</f>
         <v>0</v>
       </c>
       <c r="G4" s="31">
-        <f>lc_detailed!BL4/$X$2</f>
+        <f>lc_detailed!BM4/$W$2</f>
         <v>0</v>
       </c>
       <c r="H4" s="31">
-        <f>lc_detailed!BM4/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BN4/$W$2</f>
+        <v>0.34050656770373977</v>
       </c>
       <c r="I4" s="31">
-        <f>lc_detailed!BN4/$X$2</f>
-        <v>0.34050656770373977</v>
+        <f>lc_detailed!BO4/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J4" s="31">
-        <f>lc_detailed!BO4/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K4" s="31">
-        <f>lc_detailed!BP4/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ4/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L4" s="31">
-        <f>lc_detailed!BQ4/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR4/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M4" s="31">
-        <f>lc_detailed!BR4/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS4/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N4" s="31">
-        <f>lc_detailed!BS4/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT4/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O4" s="31">
-        <f>lc_detailed!BT4/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!CB4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P4" s="31">
-        <f>lc_detailed!CB4/$X$2</f>
+        <f>lc_detailed!CC4/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q4" s="31">
-        <f>lc_detailed!CC4/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R4" s="31">
         <f>lc_detailed!CA4</f>
         <v>0</v>
       </c>
-      <c r="S4" s="32">
+      <c r="R4" s="32">
         <f>lc_detailed!BE4</f>
         <v>499.03787819135755</v>
       </c>
-      <c r="T4" s="32">
+      <c r="S4" s="32">
         <f t="shared" si="0"/>
         <v>10.943813118231525</v>
       </c>
-      <c r="U4" s="32">
+      <c r="T4" s="32">
         <f t="shared" si="1"/>
         <v>10.943813118231525</v>
       </c>
     </row>
-    <row r="5" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="30" t="str">
+    <row r="5" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="30" t="str">
         <f>lc_detailed!AZ5</f>
         <v>CA_Ethanol_Dehydration_NGfuel</v>
       </c>
+      <c r="B5" s="31">
+        <f>lc_detailed!BH5/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C5" s="31">
-        <f>lc_detailed!BH5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI5/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D5" s="31">
-        <f>lc_detailed!BI5/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ5/$W$2</f>
+        <v>0.14502681211104032</v>
       </c>
       <c r="E5" s="31">
-        <f>lc_detailed!BJ5/$X$2</f>
-        <v>0.14502681211104032</v>
+        <f>lc_detailed!BK5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F5" s="31">
-        <f>lc_detailed!BK5/$X$2</f>
+        <f>lc_detailed!BL5/$W$2</f>
         <v>0</v>
       </c>
       <c r="G5" s="31">
-        <f>lc_detailed!BL5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BM5/$W$2</f>
+        <v>0.41273547391800947</v>
       </c>
       <c r="H5" s="31">
-        <f>lc_detailed!BM5/$X$2</f>
-        <v>0.41273547391800947</v>
+        <f>lc_detailed!BN5/$W$2</f>
+        <v>0.8288013034403614</v>
       </c>
       <c r="I5" s="31">
-        <f>lc_detailed!BN5/$X$2</f>
-        <v>0.8288013034403614</v>
+        <f>lc_detailed!BO5/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J5" s="31">
-        <f>lc_detailed!BO5/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K5" s="31">
-        <f>lc_detailed!BP5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ5/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L5" s="31">
-        <f>lc_detailed!BQ5/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR5/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M5" s="31">
-        <f>lc_detailed!BR5/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS5/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N5" s="31">
-        <f>lc_detailed!BS5/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT5/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O5" s="31">
-        <f>lc_detailed!BT5/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!CB5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P5" s="31">
-        <f>lc_detailed!CB5/$X$2</f>
+        <f>lc_detailed!CC5/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q5" s="31">
-        <f>lc_detailed!CC5/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R5" s="31">
         <f>lc_detailed!CA5</f>
         <v>0</v>
       </c>
-      <c r="S5" s="32">
+      <c r="R5" s="32">
         <f>lc_detailed!BE5</f>
         <v>525.75578125693232</v>
       </c>
-      <c r="T5" s="32">
+      <c r="S5" s="32">
         <f t="shared" si="0"/>
         <v>11.529732045108165</v>
       </c>
-      <c r="U5" s="32">
+      <c r="T5" s="32">
         <f t="shared" si="1"/>
         <v>11.529732045108165</v>
       </c>
     </row>
-    <row r="6" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="30" t="str">
+    <row r="6" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="30" t="str">
         <f>lc_detailed!AZ6</f>
         <v>CA_Ethanol_Dehydration_H2fuel</v>
       </c>
+      <c r="B6" s="31">
+        <f>lc_detailed!BH6/$W$2</f>
+        <v>0.30804920915009643</v>
+      </c>
       <c r="C6" s="31">
-        <f>lc_detailed!BH6/$X$2</f>
-        <v>0.30804920915009643</v>
+        <f>lc_detailed!BI6/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D6" s="31">
-        <f>lc_detailed!BI6/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ6/$W$2</f>
+        <v>0.14502681211104032</v>
       </c>
       <c r="E6" s="31">
-        <f>lc_detailed!BJ6/$X$2</f>
-        <v>0.14502681211104032</v>
+        <f>lc_detailed!BK6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F6" s="31">
-        <f>lc_detailed!BK6/$X$2</f>
+        <f>lc_detailed!BL6/$W$2</f>
         <v>0</v>
       </c>
       <c r="G6" s="31">
-        <f>lc_detailed!BL6/$X$2</f>
+        <f>lc_detailed!BM6/$W$2</f>
         <v>0</v>
       </c>
       <c r="H6" s="31">
-        <f>lc_detailed!BM6/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BN6/$W$2</f>
+        <v>0.8288013034403614</v>
       </c>
       <c r="I6" s="31">
-        <f>lc_detailed!BN6/$X$2</f>
-        <v>0.8288013034403614</v>
+        <f>lc_detailed!BO6/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J6" s="31">
-        <f>lc_detailed!BO6/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K6" s="31">
-        <f>lc_detailed!BP6/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ6/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L6" s="31">
-        <f>lc_detailed!BQ6/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR6/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M6" s="31">
-        <f>lc_detailed!BR6/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS6/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N6" s="31">
-        <f>lc_detailed!BS6/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT6/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O6" s="31">
-        <f>lc_detailed!BT6/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!CB6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P6" s="31">
-        <f>lc_detailed!CB6/$X$2</f>
+        <f>lc_detailed!CC6/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q6" s="31">
-        <f>lc_detailed!CC6/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R6" s="31">
         <f>lc_detailed!CA6</f>
         <v>0</v>
       </c>
-      <c r="S6" s="32">
+      <c r="R6" s="32">
         <f>lc_detailed!BE6</f>
         <v>520.98208758351552</v>
       </c>
-      <c r="T6" s="32">
+      <c r="S6" s="32">
         <f t="shared" si="0"/>
         <v>11.425045780340252</v>
       </c>
-      <c r="U6" s="32">
+      <c r="T6" s="32">
         <f t="shared" si="1"/>
         <v>11.425045780340252</v>
       </c>
     </row>
-    <row r="7" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="30" t="str">
+    <row r="7" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="30" t="str">
         <f>lc_detailed!AZ7</f>
         <v>SE_Ethanol_Dehydration_NGfuel_ethanol_biochemical</v>
       </c>
+      <c r="B7" s="31">
+        <f>lc_detailed!BH7/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C7" s="31">
-        <f>lc_detailed!BH7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI7/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D7" s="31">
-        <f>lc_detailed!BI7/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E7" s="31">
-        <f>lc_detailed!BJ7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK7/$W$2</f>
+        <v>-0.65401543344053303</v>
       </c>
       <c r="F7" s="31">
-        <f>lc_detailed!BK7/$X$2</f>
-        <v>-0.65401543344053303</v>
+        <f>lc_detailed!BL7/$W$2</f>
+        <v>11.981390717318295</v>
       </c>
       <c r="G7" s="31">
-        <f>lc_detailed!BL7/$X$2</f>
-        <v>11.981390717318295</v>
+        <f>lc_detailed!BM7/$W$2</f>
+        <v>0.16956915850640997</v>
       </c>
       <c r="H7" s="31">
-        <f>lc_detailed!BM7/$X$2</f>
-        <v>0.16956915850640997</v>
+        <f>lc_detailed!BN7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="I7" s="31">
-        <f>lc_detailed!BN7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO7/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J7" s="31">
-        <f>lc_detailed!BO7/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP7/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K7" s="31">
-        <f>lc_detailed!BP7/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ7/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L7" s="31">
-        <f>lc_detailed!BQ7/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR7/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M7" s="31">
-        <f>lc_detailed!BR7/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS7/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N7" s="31">
-        <f>lc_detailed!BS7/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT7/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O7" s="31">
-        <f>lc_detailed!BT7/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!CB7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P7" s="31">
-        <f>lc_detailed!CB7/$X$2</f>
+        <f>lc_detailed!CC7/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q7" s="31">
-        <f>lc_detailed!CC7/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R7" s="31">
         <f>lc_detailed!CA7</f>
         <v>0</v>
       </c>
-      <c r="S7" s="32">
+      <c r="R7" s="32">
         <f>lc_detailed!BE7</f>
         <v>2053.3349130738134</v>
       </c>
-      <c r="T7" s="32">
+      <c r="S7" s="32">
         <f t="shared" si="0"/>
         <v>45.029274409513448</v>
       </c>
-      <c r="U7" s="32">
+      <c r="T7" s="32">
         <f t="shared" si="1"/>
         <v>45.029274409513448</v>
       </c>
     </row>
-    <row r="8" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="30" t="str">
+    <row r="8" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="30" t="str">
         <f>lc_detailed!AZ8</f>
         <v>SE_Ethanol_Dehydration_H2fuel_ethanol_biochemical</v>
       </c>
+      <c r="B8" s="31">
+        <f>lc_detailed!BH8/$W$2</f>
+        <v>0.30171339336527736</v>
+      </c>
       <c r="C8" s="31">
-        <f>lc_detailed!BH8/$X$2</f>
-        <v>0.30171339336527736</v>
+        <f>lc_detailed!BI8/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D8" s="31">
-        <f>lc_detailed!BI8/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E8" s="31">
-        <f>lc_detailed!BJ8/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK8/$W$2</f>
+        <v>-0.65401543344053303</v>
       </c>
       <c r="F8" s="31">
-        <f>lc_detailed!BK8/$X$2</f>
-        <v>-0.65401543344053303</v>
+        <f>lc_detailed!BL8/$W$2</f>
+        <v>11.981390717318295</v>
       </c>
       <c r="G8" s="31">
-        <f>lc_detailed!BL8/$X$2</f>
-        <v>11.981390717318295</v>
+        <f>lc_detailed!BM8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="H8" s="31">
-        <f>lc_detailed!BM8/$X$2</f>
+        <f>lc_detailed!BN8/$W$2</f>
         <v>0</v>
       </c>
       <c r="I8" s="31">
-        <f>lc_detailed!BN8/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO8/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J8" s="31">
-        <f>lc_detailed!BO8/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP8/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K8" s="31">
-        <f>lc_detailed!BP8/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ8/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L8" s="31">
-        <f>lc_detailed!BQ8/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR8/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M8" s="31">
-        <f>lc_detailed!BR8/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS8/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N8" s="31">
-        <f>lc_detailed!BS8/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT8/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O8" s="31">
-        <f>lc_detailed!BT8/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!CB8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P8" s="31">
-        <f>lc_detailed!CB8/$X$2</f>
+        <f>lc_detailed!CC8/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q8" s="31">
-        <f>lc_detailed!CC8/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R8" s="31">
         <f>lc_detailed!CA8</f>
         <v>0</v>
       </c>
-      <c r="S8" s="32">
+      <c r="R8" s="32">
         <f>lc_detailed!BE8</f>
         <v>2059.3606901833773</v>
       </c>
-      <c r="T8" s="32">
+      <c r="S8" s="32">
         <f t="shared" si="0"/>
         <v>45.161418644372311</v>
       </c>
-      <c r="U8" s="32">
+      <c r="T8" s="32">
         <f t="shared" si="1"/>
         <v>45.161418644372318</v>
       </c>
     </row>
-    <row r="9" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="30" t="str">
+    <row r="9" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="30" t="str">
         <f>lc_detailed!AZ9</f>
         <v>CA_Ethanol_Dehydration_NGfuel_ethanol_biochemical</v>
       </c>
+      <c r="B9" s="31">
+        <f>lc_detailed!BH9/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C9" s="31">
-        <f>lc_detailed!BH9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI9/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D9" s="31">
-        <f>lc_detailed!BI9/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E9" s="31">
-        <f>lc_detailed!BJ9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK9/$W$2</f>
+        <v>-0.62341237236486724</v>
       </c>
       <c r="F9" s="31">
-        <f>lc_detailed!BK9/$X$2</f>
-        <v>-0.62341237236486724</v>
+        <f>lc_detailed!BL9/$W$2</f>
+        <v>14.614183152615643</v>
       </c>
       <c r="G9" s="31">
-        <f>lc_detailed!BL9/$X$2</f>
-        <v>14.614183152615643</v>
+        <f>lc_detailed!BM9/$W$2</f>
+        <v>0.41273547391800947</v>
       </c>
       <c r="H9" s="31">
-        <f>lc_detailed!BM9/$X$2</f>
-        <v>0.41273547391800947</v>
+        <f>lc_detailed!BN9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="I9" s="31">
-        <f>lc_detailed!BN9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO9/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J9" s="31">
-        <f>lc_detailed!BO9/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP9/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K9" s="31">
-        <f>lc_detailed!BP9/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ9/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L9" s="31">
-        <f>lc_detailed!BQ9/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR9/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M9" s="31">
-        <f>lc_detailed!BR9/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS9/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N9" s="31">
-        <f>lc_detailed!BS9/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT9/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O9" s="31">
-        <f>lc_detailed!BT9/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!CB9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P9" s="31">
-        <f>lc_detailed!CB9/$X$2</f>
+        <f>lc_detailed!CC9/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q9" s="31">
-        <f>lc_detailed!CC9/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R9" s="31">
         <f>lc_detailed!CA9</f>
         <v>0</v>
       </c>
-      <c r="S9" s="32">
+      <c r="R9" s="32">
         <f>lc_detailed!BE9</f>
         <v>2185.5878283567381</v>
       </c>
-      <c r="T9" s="32">
+      <c r="S9" s="32">
         <f t="shared" si="0"/>
         <v>47.929557639402148</v>
       </c>
-      <c r="U9" s="32">
+      <c r="T9" s="32">
         <f t="shared" si="1"/>
         <v>47.929557639402148</v>
       </c>
     </row>
-    <row r="10" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="30" t="str">
+    <row r="10" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="30" t="str">
         <f>lc_detailed!AZ10</f>
         <v>CA_Ethanol_Dehydration_H2fuel_ethanol_biochemical</v>
       </c>
+      <c r="B10" s="31">
+        <f>lc_detailed!BH10/$W$2</f>
+        <v>0.30804920915009643</v>
+      </c>
       <c r="C10" s="31">
-        <f>lc_detailed!BH10/$X$2</f>
-        <v>0.30804920915009643</v>
+        <f>lc_detailed!BI10/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D10" s="31">
-        <f>lc_detailed!BI10/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E10" s="31">
-        <f>lc_detailed!BJ10/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK10/$W$2</f>
+        <v>-0.62341237236486724</v>
       </c>
       <c r="F10" s="31">
-        <f>lc_detailed!BK10/$X$2</f>
-        <v>-0.62341237236486724</v>
+        <f>lc_detailed!BL10/$W$2</f>
+        <v>14.614183152615643</v>
       </c>
       <c r="G10" s="31">
-        <f>lc_detailed!BL10/$X$2</f>
-        <v>14.614183152615643</v>
+        <f>lc_detailed!BM10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="H10" s="31">
-        <f>lc_detailed!BM10/$X$2</f>
+        <f>lc_detailed!BN10/$W$2</f>
         <v>0</v>
       </c>
       <c r="I10" s="31">
-        <f>lc_detailed!BN10/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO10/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J10" s="31">
-        <f>lc_detailed!BO10/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP10/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K10" s="31">
-        <f>lc_detailed!BP10/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ10/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L10" s="31">
-        <f>lc_detailed!BQ10/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR10/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M10" s="31">
-        <f>lc_detailed!BR10/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS10/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N10" s="31">
-        <f>lc_detailed!BS10/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT10/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O10" s="31">
-        <f>lc_detailed!BT10/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!CB10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P10" s="31">
-        <f>lc_detailed!CB10/$X$2</f>
+        <f>lc_detailed!CC10/$W$2</f>
         <v>0</v>
       </c>
       <c r="Q10" s="31">
-        <f>lc_detailed!CC10/$X$2</f>
-        <v>0</v>
-      </c>
-      <c r="R10" s="31">
         <f>lc_detailed!CA10</f>
         <v>0</v>
       </c>
-      <c r="S10" s="32">
+      <c r="R10" s="32">
         <f>lc_detailed!BE10</f>
         <v>2180.8141346833208</v>
       </c>
-      <c r="T10" s="32">
+      <c r="S10" s="32">
         <f t="shared" si="0"/>
         <v>47.824871374634228</v>
       </c>
-      <c r="U10" s="32">
+      <c r="T10" s="32">
         <f t="shared" si="1"/>
         <v>47.824871374634235</v>
       </c>
     </row>
-    <row r="11" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="30"/>
+    <row r="11" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
       <c r="C11" s="31"/>
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
@@ -9648,13 +9648,13 @@
       <c r="O11" s="31"/>
       <c r="P11" s="31"/>
       <c r="Q11" s="31"/>
-      <c r="R11" s="31"/>
+      <c r="R11" s="32"/>
       <c r="S11" s="32"/>
       <c r="T11" s="32"/>
-      <c r="U11" s="32"/>
-    </row>
-    <row r="12" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="30"/>
+    </row>
+    <row r="12" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
@@ -9670,13 +9670,13 @@
       <c r="O12" s="31"/>
       <c r="P12" s="31"/>
       <c r="Q12" s="31"/>
-      <c r="R12" s="31"/>
+      <c r="R12" s="32"/>
       <c r="S12" s="32"/>
       <c r="T12" s="32"/>
-      <c r="U12" s="32"/>
-    </row>
-    <row r="13" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="30"/>
+    </row>
+    <row r="13" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="30"/>
+      <c r="B13" s="31"/>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
       <c r="E13" s="31"/>
@@ -9692,13 +9692,13 @@
       <c r="O13" s="31"/>
       <c r="P13" s="31"/>
       <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
+      <c r="R13" s="32"/>
       <c r="S13" s="32"/>
       <c r="T13" s="32"/>
-      <c r="U13" s="32"/>
-    </row>
-    <row r="14" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="30"/>
+    </row>
+    <row r="14" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="30"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
       <c r="E14" s="31"/>
@@ -9714,13 +9714,13 @@
       <c r="O14" s="31"/>
       <c r="P14" s="31"/>
       <c r="Q14" s="31"/>
-      <c r="R14" s="31"/>
+      <c r="R14" s="32"/>
       <c r="S14" s="32"/>
       <c r="T14" s="32"/>
-      <c r="U14" s="32"/>
-    </row>
-    <row r="15" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="30"/>
+    </row>
+    <row r="15" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="30"/>
+      <c r="B15" s="31"/>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
@@ -9736,13 +9736,13 @@
       <c r="O15" s="31"/>
       <c r="P15" s="31"/>
       <c r="Q15" s="31"/>
-      <c r="R15" s="31"/>
+      <c r="R15" s="32"/>
       <c r="S15" s="32"/>
       <c r="T15" s="32"/>
-      <c r="U15" s="32"/>
-    </row>
-    <row r="16" spans="2:25" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="30"/>
+    </row>
+    <row r="16" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
@@ -9758,13 +9758,13 @@
       <c r="O16" s="31"/>
       <c r="P16" s="31"/>
       <c r="Q16" s="31"/>
-      <c r="R16" s="31"/>
+      <c r="R16" s="32"/>
       <c r="S16" s="32"/>
       <c r="T16" s="32"/>
-      <c r="U16" s="32"/>
-    </row>
-    <row r="17" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="30"/>
+    </row>
+    <row r="17" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="30"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="31"/>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
@@ -9780,13 +9780,13 @@
       <c r="O17" s="31"/>
       <c r="P17" s="31"/>
       <c r="Q17" s="31"/>
-      <c r="R17" s="31"/>
+      <c r="R17" s="32"/>
       <c r="S17" s="32"/>
       <c r="T17" s="32"/>
-      <c r="U17" s="32"/>
-    </row>
-    <row r="18" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="30"/>
+    </row>
+    <row r="18" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="30"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
@@ -9802,13 +9802,13 @@
       <c r="O18" s="31"/>
       <c r="P18" s="31"/>
       <c r="Q18" s="31"/>
-      <c r="R18" s="31"/>
+      <c r="R18" s="32"/>
       <c r="S18" s="32"/>
       <c r="T18" s="32"/>
-      <c r="U18" s="32"/>
-    </row>
-    <row r="19" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="30"/>
+    </row>
+    <row r="19" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="30"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="31"/>
       <c r="D19" s="31"/>
       <c r="E19" s="31"/>
@@ -9824,13 +9824,13 @@
       <c r="O19" s="31"/>
       <c r="P19" s="31"/>
       <c r="Q19" s="31"/>
-      <c r="R19" s="31"/>
+      <c r="R19" s="32"/>
       <c r="S19" s="32"/>
       <c r="T19" s="32"/>
-      <c r="U19" s="32"/>
-    </row>
-    <row r="20" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="30"/>
+    </row>
+    <row r="20" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="30"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="31"/>
       <c r="D20" s="31"/>
       <c r="E20" s="31"/>
@@ -9846,13 +9846,13 @@
       <c r="O20" s="31"/>
       <c r="P20" s="31"/>
       <c r="Q20" s="31"/>
-      <c r="R20" s="31"/>
+      <c r="R20" s="32"/>
       <c r="S20" s="32"/>
       <c r="T20" s="32"/>
-      <c r="U20" s="32"/>
-    </row>
-    <row r="21" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="30"/>
+    </row>
+    <row r="21" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="30"/>
+      <c r="B21" s="31"/>
       <c r="C21" s="31"/>
       <c r="D21" s="31"/>
       <c r="E21" s="31"/>
@@ -9868,13 +9868,13 @@
       <c r="O21" s="31"/>
       <c r="P21" s="31"/>
       <c r="Q21" s="31"/>
-      <c r="R21" s="31"/>
+      <c r="R21" s="32"/>
       <c r="S21" s="32"/>
       <c r="T21" s="32"/>
-      <c r="U21" s="32"/>
-    </row>
-    <row r="22" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="30"/>
+    </row>
+    <row r="22" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="31"/>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -9890,13 +9890,13 @@
       <c r="O22" s="31"/>
       <c r="P22" s="31"/>
       <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
+      <c r="R22" s="32"/>
       <c r="S22" s="32"/>
       <c r="T22" s="32"/>
-      <c r="U22" s="32"/>
-    </row>
-    <row r="23" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="30"/>
+    </row>
+    <row r="23" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="30"/>
+      <c r="B23" s="31"/>
       <c r="C23" s="31"/>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -9912,13 +9912,13 @@
       <c r="O23" s="31"/>
       <c r="P23" s="31"/>
       <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
+      <c r="R23" s="32"/>
       <c r="S23" s="32"/>
       <c r="T23" s="32"/>
-      <c r="U23" s="32"/>
-    </row>
-    <row r="24" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="30"/>
+    </row>
+    <row r="24" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="30"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="31"/>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -9934,13 +9934,13 @@
       <c r="O24" s="31"/>
       <c r="P24" s="31"/>
       <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
+      <c r="R24" s="32"/>
       <c r="S24" s="32"/>
       <c r="T24" s="32"/>
-      <c r="U24" s="32"/>
-    </row>
-    <row r="25" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="30"/>
+    </row>
+    <row r="25" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="30"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="31"/>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -9956,13 +9956,13 @@
       <c r="O25" s="31"/>
       <c r="P25" s="31"/>
       <c r="Q25" s="31"/>
-      <c r="R25" s="31"/>
+      <c r="R25" s="32"/>
       <c r="S25" s="32"/>
       <c r="T25" s="32"/>
-      <c r="U25" s="32"/>
-    </row>
-    <row r="26" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="30"/>
+    </row>
+    <row r="26" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="30"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="31"/>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -9978,13 +9978,13 @@
       <c r="O26" s="31"/>
       <c r="P26" s="31"/>
       <c r="Q26" s="31"/>
-      <c r="R26" s="31"/>
+      <c r="R26" s="32"/>
       <c r="S26" s="32"/>
       <c r="T26" s="32"/>
-      <c r="U26" s="32"/>
-    </row>
-    <row r="27" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="30"/>
+    </row>
+    <row r="27" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="30"/>
+      <c r="B27" s="31"/>
       <c r="C27" s="31"/>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -10000,13 +10000,13 @@
       <c r="O27" s="31"/>
       <c r="P27" s="31"/>
       <c r="Q27" s="31"/>
-      <c r="R27" s="31"/>
+      <c r="R27" s="32"/>
       <c r="S27" s="32"/>
       <c r="T27" s="32"/>
-      <c r="U27" s="32"/>
-    </row>
-    <row r="28" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="30"/>
+    </row>
+    <row r="28" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="30"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
       <c r="E28" s="31"/>
@@ -10022,13 +10022,13 @@
       <c r="O28" s="31"/>
       <c r="P28" s="31"/>
       <c r="Q28" s="31"/>
-      <c r="R28" s="31"/>
+      <c r="R28" s="32"/>
       <c r="S28" s="32"/>
       <c r="T28" s="32"/>
-      <c r="U28" s="32"/>
-    </row>
-    <row r="29" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="30"/>
+    </row>
+    <row r="29" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="30"/>
+      <c r="B29" s="31"/>
       <c r="C29" s="31"/>
       <c r="D29" s="31"/>
       <c r="E29" s="31"/>
@@ -10044,13 +10044,13 @@
       <c r="O29" s="31"/>
       <c r="P29" s="31"/>
       <c r="Q29" s="31"/>
-      <c r="R29" s="31"/>
+      <c r="R29" s="32"/>
       <c r="S29" s="32"/>
       <c r="T29" s="32"/>
-      <c r="U29" s="32"/>
-    </row>
-    <row r="30" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="30"/>
+    </row>
+    <row r="30" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="30"/>
+      <c r="B30" s="31"/>
       <c r="C30" s="31"/>
       <c r="D30" s="31"/>
       <c r="E30" s="31"/>
@@ -10066,13 +10066,13 @@
       <c r="O30" s="31"/>
       <c r="P30" s="31"/>
       <c r="Q30" s="31"/>
-      <c r="R30" s="31"/>
+      <c r="R30" s="32"/>
       <c r="S30" s="32"/>
       <c r="T30" s="32"/>
-      <c r="U30" s="32"/>
-    </row>
-    <row r="31" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="30"/>
+    </row>
+    <row r="31" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="30"/>
+      <c r="B31" s="31"/>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
       <c r="E31" s="31"/>
@@ -10088,13 +10088,13 @@
       <c r="O31" s="31"/>
       <c r="P31" s="31"/>
       <c r="Q31" s="31"/>
-      <c r="R31" s="31"/>
+      <c r="R31" s="32"/>
       <c r="S31" s="32"/>
       <c r="T31" s="32"/>
-      <c r="U31" s="32"/>
-    </row>
-    <row r="32" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="30"/>
+    </row>
+    <row r="32" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="30"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="31"/>
       <c r="D32" s="31"/>
       <c r="E32" s="31"/>
@@ -10110,13 +10110,13 @@
       <c r="O32" s="31"/>
       <c r="P32" s="31"/>
       <c r="Q32" s="31"/>
-      <c r="R32" s="31"/>
+      <c r="R32" s="32"/>
       <c r="S32" s="32"/>
       <c r="T32" s="32"/>
-      <c r="U32" s="32"/>
-    </row>
-    <row r="33" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="30"/>
+    </row>
+    <row r="33" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="30"/>
+      <c r="B33" s="31"/>
       <c r="C33" s="31"/>
       <c r="D33" s="31"/>
       <c r="E33" s="31"/>
@@ -10132,13 +10132,13 @@
       <c r="O33" s="31"/>
       <c r="P33" s="31"/>
       <c r="Q33" s="31"/>
-      <c r="R33" s="31"/>
+      <c r="R33" s="32"/>
       <c r="S33" s="32"/>
       <c r="T33" s="32"/>
-      <c r="U33" s="32"/>
-    </row>
-    <row r="34" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="30"/>
+    </row>
+    <row r="34" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="30"/>
+      <c r="B34" s="31"/>
       <c r="C34" s="31"/>
       <c r="D34" s="31"/>
       <c r="E34" s="31"/>
@@ -10154,13 +10154,13 @@
       <c r="O34" s="31"/>
       <c r="P34" s="31"/>
       <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
+      <c r="R34" s="32"/>
       <c r="S34" s="32"/>
       <c r="T34" s="32"/>
-      <c r="U34" s="32"/>
-    </row>
-    <row r="35" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="30"/>
+    </row>
+    <row r="35" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="30"/>
+      <c r="B35" s="31"/>
       <c r="C35" s="31"/>
       <c r="D35" s="31"/>
       <c r="E35" s="31"/>
@@ -10176,13 +10176,13 @@
       <c r="O35" s="31"/>
       <c r="P35" s="31"/>
       <c r="Q35" s="31"/>
-      <c r="R35" s="31"/>
+      <c r="R35" s="32"/>
       <c r="S35" s="32"/>
       <c r="T35" s="32"/>
-      <c r="U35" s="32"/>
-    </row>
-    <row r="36" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="30"/>
+    </row>
+    <row r="36" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="30"/>
+      <c r="B36" s="31"/>
       <c r="C36" s="31"/>
       <c r="D36" s="31"/>
       <c r="E36" s="31"/>
@@ -10198,13 +10198,13 @@
       <c r="O36" s="31"/>
       <c r="P36" s="31"/>
       <c r="Q36" s="31"/>
-      <c r="R36" s="31"/>
+      <c r="R36" s="32"/>
       <c r="S36" s="32"/>
       <c r="T36" s="32"/>
-      <c r="U36" s="32"/>
-    </row>
-    <row r="37" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="30"/>
+    </row>
+    <row r="37" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="30"/>
+      <c r="B37" s="31"/>
       <c r="C37" s="31"/>
       <c r="D37" s="31"/>
       <c r="E37" s="31"/>
@@ -10220,13 +10220,13 @@
       <c r="O37" s="31"/>
       <c r="P37" s="31"/>
       <c r="Q37" s="31"/>
-      <c r="R37" s="31"/>
+      <c r="R37" s="32"/>
       <c r="S37" s="32"/>
       <c r="T37" s="32"/>
-      <c r="U37" s="32"/>
-    </row>
-    <row r="38" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="30"/>
+    </row>
+    <row r="38" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="30"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="31"/>
       <c r="D38" s="31"/>
       <c r="E38" s="31"/>
@@ -10242,13 +10242,13 @@
       <c r="O38" s="31"/>
       <c r="P38" s="31"/>
       <c r="Q38" s="31"/>
-      <c r="R38" s="31"/>
+      <c r="R38" s="32"/>
       <c r="S38" s="32"/>
       <c r="T38" s="32"/>
-      <c r="U38" s="32"/>
-    </row>
-    <row r="39" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="30"/>
+    </row>
+    <row r="39" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="30"/>
+      <c r="B39" s="31"/>
       <c r="C39" s="31"/>
       <c r="D39" s="31"/>
       <c r="E39" s="31"/>
@@ -10264,13 +10264,13 @@
       <c r="O39" s="31"/>
       <c r="P39" s="31"/>
       <c r="Q39" s="31"/>
-      <c r="R39" s="31"/>
+      <c r="R39" s="32"/>
       <c r="S39" s="32"/>
       <c r="T39" s="32"/>
-      <c r="U39" s="32"/>
-    </row>
-    <row r="40" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="30"/>
+    </row>
+    <row r="40" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="30"/>
+      <c r="B40" s="31"/>
       <c r="C40" s="31"/>
       <c r="D40" s="31"/>
       <c r="E40" s="31"/>
@@ -10286,13 +10286,13 @@
       <c r="O40" s="31"/>
       <c r="P40" s="31"/>
       <c r="Q40" s="31"/>
-      <c r="R40" s="31"/>
+      <c r="R40" s="32"/>
       <c r="S40" s="32"/>
       <c r="T40" s="32"/>
-      <c r="U40" s="32"/>
-    </row>
-    <row r="41" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="30"/>
+    </row>
+    <row r="41" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="30"/>
+      <c r="B41" s="31"/>
       <c r="C41" s="31"/>
       <c r="D41" s="31"/>
       <c r="E41" s="31"/>
@@ -10308,13 +10308,13 @@
       <c r="O41" s="31"/>
       <c r="P41" s="31"/>
       <c r="Q41" s="31"/>
-      <c r="R41" s="31"/>
+      <c r="R41" s="32"/>
       <c r="S41" s="32"/>
       <c r="T41" s="32"/>
-      <c r="U41" s="32"/>
-    </row>
-    <row r="42" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="30"/>
+    </row>
+    <row r="42" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="30"/>
+      <c r="B42" s="31"/>
       <c r="C42" s="31"/>
       <c r="D42" s="31"/>
       <c r="E42" s="31"/>
@@ -10330,13 +10330,13 @@
       <c r="O42" s="31"/>
       <c r="P42" s="31"/>
       <c r="Q42" s="31"/>
-      <c r="R42" s="31"/>
+      <c r="R42" s="32"/>
       <c r="S42" s="32"/>
       <c r="T42" s="32"/>
-      <c r="U42" s="32"/>
-    </row>
-    <row r="43" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="30"/>
+    </row>
+    <row r="43" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="30"/>
+      <c r="B43" s="31"/>
       <c r="C43" s="31"/>
       <c r="D43" s="31"/>
       <c r="E43" s="31"/>
@@ -10352,13 +10352,13 @@
       <c r="O43" s="31"/>
       <c r="P43" s="31"/>
       <c r="Q43" s="31"/>
-      <c r="R43" s="31"/>
+      <c r="R43" s="32"/>
       <c r="S43" s="32"/>
       <c r="T43" s="32"/>
-      <c r="U43" s="32"/>
-    </row>
-    <row r="44" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="30"/>
+    </row>
+    <row r="44" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="30"/>
+      <c r="B44" s="31"/>
       <c r="C44" s="31"/>
       <c r="D44" s="31"/>
       <c r="E44" s="31"/>
@@ -10374,13 +10374,13 @@
       <c r="O44" s="31"/>
       <c r="P44" s="31"/>
       <c r="Q44" s="31"/>
-      <c r="R44" s="31"/>
+      <c r="R44" s="32"/>
       <c r="S44" s="32"/>
       <c r="T44" s="32"/>
-      <c r="U44" s="32"/>
-    </row>
-    <row r="45" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="30"/>
+    </row>
+    <row r="45" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="30"/>
+      <c r="B45" s="31"/>
       <c r="C45" s="31"/>
       <c r="D45" s="31"/>
       <c r="E45" s="31"/>
@@ -10396,13 +10396,13 @@
       <c r="O45" s="31"/>
       <c r="P45" s="31"/>
       <c r="Q45" s="31"/>
-      <c r="R45" s="31"/>
+      <c r="R45" s="32"/>
       <c r="S45" s="32"/>
       <c r="T45" s="32"/>
-      <c r="U45" s="32"/>
-    </row>
-    <row r="46" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="30"/>
+    </row>
+    <row r="46" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="30"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="31"/>
       <c r="D46" s="31"/>
       <c r="E46" s="31"/>
@@ -10418,13 +10418,13 @@
       <c r="O46" s="31"/>
       <c r="P46" s="31"/>
       <c r="Q46" s="31"/>
-      <c r="R46" s="31"/>
+      <c r="R46" s="32"/>
       <c r="S46" s="32"/>
       <c r="T46" s="32"/>
-      <c r="U46" s="32"/>
-    </row>
-    <row r="47" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="30"/>
+    </row>
+    <row r="47" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="30"/>
+      <c r="B47" s="31"/>
       <c r="C47" s="31"/>
       <c r="D47" s="31"/>
       <c r="E47" s="31"/>
@@ -10440,13 +10440,13 @@
       <c r="O47" s="31"/>
       <c r="P47" s="31"/>
       <c r="Q47" s="31"/>
-      <c r="R47" s="31"/>
+      <c r="R47" s="32"/>
       <c r="S47" s="32"/>
       <c r="T47" s="32"/>
-      <c r="U47" s="32"/>
-    </row>
-    <row r="48" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="30"/>
+    </row>
+    <row r="48" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="30"/>
+      <c r="B48" s="31"/>
       <c r="C48" s="31"/>
       <c r="D48" s="31"/>
       <c r="E48" s="31"/>
@@ -10462,13 +10462,13 @@
       <c r="O48" s="31"/>
       <c r="P48" s="31"/>
       <c r="Q48" s="31"/>
-      <c r="R48" s="31"/>
+      <c r="R48" s="32"/>
       <c r="S48" s="32"/>
       <c r="T48" s="32"/>
-      <c r="U48" s="32"/>
-    </row>
-    <row r="49" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="30"/>
+    </row>
+    <row r="49" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="30"/>
+      <c r="B49" s="31"/>
       <c r="C49" s="31"/>
       <c r="D49" s="31"/>
       <c r="E49" s="31"/>
@@ -10484,13 +10484,13 @@
       <c r="O49" s="31"/>
       <c r="P49" s="31"/>
       <c r="Q49" s="31"/>
-      <c r="R49" s="31"/>
+      <c r="R49" s="32"/>
       <c r="S49" s="32"/>
       <c r="T49" s="32"/>
-      <c r="U49" s="32"/>
-    </row>
-    <row r="50" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="30"/>
+    </row>
+    <row r="50" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="30"/>
+      <c r="B50" s="31"/>
       <c r="C50" s="31"/>
       <c r="D50" s="31"/>
       <c r="E50" s="31"/>
@@ -10506,13 +10506,13 @@
       <c r="O50" s="31"/>
       <c r="P50" s="31"/>
       <c r="Q50" s="31"/>
-      <c r="R50" s="31"/>
+      <c r="R50" s="32"/>
       <c r="S50" s="32"/>
       <c r="T50" s="32"/>
-      <c r="U50" s="32"/>
-    </row>
-    <row r="51" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="30"/>
+    </row>
+    <row r="51" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="30"/>
+      <c r="B51" s="31"/>
       <c r="C51" s="31"/>
       <c r="D51" s="31"/>
       <c r="E51" s="31"/>
@@ -10528,13 +10528,13 @@
       <c r="O51" s="31"/>
       <c r="P51" s="31"/>
       <c r="Q51" s="31"/>
-      <c r="R51" s="31"/>
+      <c r="R51" s="32"/>
       <c r="S51" s="32"/>
       <c r="T51" s="32"/>
-      <c r="U51" s="32"/>
-    </row>
-    <row r="52" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B52" s="30"/>
+    </row>
+    <row r="52" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="30"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="31"/>
       <c r="D52" s="31"/>
       <c r="E52" s="31"/>
@@ -10550,13 +10550,13 @@
       <c r="O52" s="31"/>
       <c r="P52" s="31"/>
       <c r="Q52" s="31"/>
-      <c r="R52" s="31"/>
+      <c r="R52" s="32"/>
       <c r="S52" s="32"/>
       <c r="T52" s="32"/>
-      <c r="U52" s="32"/>
-    </row>
-    <row r="53" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="30"/>
+    </row>
+    <row r="53" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="30"/>
+      <c r="B53" s="31"/>
       <c r="C53" s="31"/>
       <c r="D53" s="31"/>
       <c r="E53" s="31"/>
@@ -10572,13 +10572,13 @@
       <c r="O53" s="31"/>
       <c r="P53" s="31"/>
       <c r="Q53" s="31"/>
-      <c r="R53" s="31"/>
+      <c r="R53" s="32"/>
       <c r="S53" s="32"/>
       <c r="T53" s="32"/>
-      <c r="U53" s="32"/>
-    </row>
-    <row r="54" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="30"/>
+    </row>
+    <row r="54" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="30"/>
+      <c r="B54" s="31"/>
       <c r="C54" s="31"/>
       <c r="D54" s="31"/>
       <c r="E54" s="31"/>
@@ -10594,13 +10594,13 @@
       <c r="O54" s="31"/>
       <c r="P54" s="31"/>
       <c r="Q54" s="31"/>
-      <c r="R54" s="31"/>
+      <c r="R54" s="32"/>
       <c r="S54" s="32"/>
       <c r="T54" s="32"/>
-      <c r="U54" s="32"/>
-    </row>
-    <row r="55" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="30"/>
+    </row>
+    <row r="55" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="30"/>
+      <c r="B55" s="31"/>
       <c r="C55" s="31"/>
       <c r="D55" s="31"/>
       <c r="E55" s="31"/>
@@ -10616,13 +10616,13 @@
       <c r="O55" s="31"/>
       <c r="P55" s="31"/>
       <c r="Q55" s="31"/>
-      <c r="R55" s="31"/>
+      <c r="R55" s="32"/>
       <c r="S55" s="32"/>
       <c r="T55" s="32"/>
-      <c r="U55" s="32"/>
-    </row>
-    <row r="56" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="30"/>
+    </row>
+    <row r="56" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="30"/>
+      <c r="B56" s="31"/>
       <c r="C56" s="31"/>
       <c r="D56" s="31"/>
       <c r="E56" s="31"/>
@@ -10638,13 +10638,13 @@
       <c r="O56" s="31"/>
       <c r="P56" s="31"/>
       <c r="Q56" s="31"/>
-      <c r="R56" s="31"/>
+      <c r="R56" s="32"/>
       <c r="S56" s="32"/>
       <c r="T56" s="32"/>
-      <c r="U56" s="32"/>
-    </row>
-    <row r="57" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="30"/>
+    </row>
+    <row r="57" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="30"/>
+      <c r="B57" s="31"/>
       <c r="C57" s="31"/>
       <c r="D57" s="31"/>
       <c r="E57" s="31"/>
@@ -10660,13 +10660,13 @@
       <c r="O57" s="31"/>
       <c r="P57" s="31"/>
       <c r="Q57" s="31"/>
-      <c r="R57" s="31"/>
+      <c r="R57" s="32"/>
       <c r="S57" s="32"/>
       <c r="T57" s="32"/>
-      <c r="U57" s="32"/>
-    </row>
-    <row r="58" spans="2:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="30"/>
+    </row>
+    <row r="58" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="30"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="31"/>
       <c r="D58" s="31"/>
       <c r="E58" s="31"/>
@@ -10682,10 +10682,9 @@
       <c r="O58" s="31"/>
       <c r="P58" s="31"/>
       <c r="Q58" s="31"/>
-      <c r="R58" s="31"/>
+      <c r="R58" s="32"/>
       <c r="S58" s="32"/>
       <c r="T58" s="32"/>
-      <c r="U58" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10694,804 +10693,804 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:Y27"/>
+  <dimension ref="A1:X27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.5" customWidth="1"/>
-    <col min="2" max="2" width="49.1640625" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.6640625" customWidth="1"/>
-    <col min="14" max="14" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.83203125" customWidth="1"/>
-    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" customWidth="1"/>
-    <col min="18" max="18" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="2.6640625" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.1640625" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.6640625" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="2.6640625" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B1" s="21" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="W1" s="28" t="s">
+      <c r="V1" s="28" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="2:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="23" t="s">
+        <v>68</v>
+      </c>
       <c r="B2" s="23" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="O2" s="23" t="s">
         <v>84</v>
       </c>
+      <c r="O2" s="24" t="s">
+        <v>86</v>
+      </c>
       <c r="P2" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q2" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="R2" s="24" t="s">
         <v>85</v>
       </c>
+      <c r="R2" s="25" t="s">
+        <v>70</v>
+      </c>
       <c r="S2" s="25" t="s">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="T2" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="U2" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="W2" t="s">
+      <c r="V2" t="s">
         <v>126</v>
       </c>
-      <c r="X2">
+      <c r="W2">
         <v>45.6</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="X2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B3" t="str">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A3" t="str">
         <f>lc_detailed!AZ3</f>
         <v>SE_Ethanol_Dehydration_NGfuel</v>
       </c>
+      <c r="B3" s="29">
+        <f>lc_detailed!BH3/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C3" s="29">
-        <f>lc_detailed!BH3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI3/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D3" s="29">
-        <f>lc_detailed!BI3/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ3/$W$2</f>
+        <v>0.15214611962784025</v>
       </c>
       <c r="E3" s="29">
-        <f>lc_detailed!BJ3/$X$2</f>
-        <v>0.15214611962784025</v>
+        <f>lc_detailed!BK3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F3" s="29">
-        <f>lc_detailed!BK3/$X$2</f>
+        <f>lc_detailed!BL3/$W$2</f>
         <v>0</v>
       </c>
       <c r="G3" s="29">
-        <f>lc_detailed!BL3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BM3/$W$2</f>
+        <v>0.16956915850640997</v>
       </c>
       <c r="H3" s="29">
-        <f>lc_detailed!BM3/$X$2</f>
-        <v>0.16956915850640997</v>
+        <f>lc_detailed!BN3/$W$2</f>
+        <v>0.34050656770373977</v>
       </c>
       <c r="I3" s="29">
-        <f>lc_detailed!BN3/$X$2</f>
-        <v>0.34050656770373977</v>
+        <f>lc_detailed!BO3/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J3" s="29">
-        <f>lc_detailed!BO3/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K3" s="29">
-        <f>lc_detailed!BP3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ3/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L3" s="29">
-        <f>lc_detailed!BQ3/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR3/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M3" s="29">
-        <f>lc_detailed!BR3/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS3/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N3" s="29">
-        <f>lc_detailed!BS3/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT3/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O3" s="29">
-        <f>lc_detailed!BT3/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!BV3/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P3" s="29">
-        <f>lc_detailed!BV3/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW3/$W$2</f>
+        <v>-8.4102014092105168</v>
       </c>
       <c r="Q3" s="29">
-        <f>lc_detailed!BW3/$X$2</f>
-        <v>-8.4102014092105168</v>
-      </c>
-      <c r="R3" s="29">
         <f>lc_detailed!BU3</f>
         <v>-3.1399999999999966</v>
       </c>
-      <c r="S3" s="29">
+      <c r="R3" s="29">
         <f>lc_detailed!BB3</f>
         <v>109.5069168217936</v>
       </c>
+      <c r="S3" s="29">
+        <f t="shared" ref="S3:S10" si="0">R3/$W$2</f>
+        <v>2.40146747416214</v>
+      </c>
       <c r="T3" s="29">
-        <f t="shared" ref="T3:T10" si="0">S3/$X$2</f>
-        <v>2.40146747416214</v>
-      </c>
-      <c r="U3" s="29">
-        <f t="shared" ref="U3:U10" si="1">SUM(C3:Q3)</f>
+        <f t="shared" ref="T3:T10" si="1">SUM(B3:P3)</f>
         <v>2.4014674741621409</v>
       </c>
+      <c r="U3" s="29"/>
       <c r="V3" s="29"/>
       <c r="W3" s="29"/>
       <c r="X3" s="29"/>
-      <c r="Y3" s="29"/>
-    </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B4" t="str">
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A4" t="str">
         <f>lc_detailed!AZ4</f>
         <v>SE_Ethanol_Dehydration_H2fuel</v>
       </c>
+      <c r="B4" s="29">
+        <f>lc_detailed!BH4/$W$2</f>
+        <v>0.30171339336527736</v>
+      </c>
       <c r="C4" s="29">
-        <f>lc_detailed!BH4/$X$2</f>
-        <v>0.30171339336527736</v>
+        <f>lc_detailed!BI4/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D4" s="29">
-        <f>lc_detailed!BI4/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ4/$W$2</f>
+        <v>0.15214611962784025</v>
       </c>
       <c r="E4" s="29">
-        <f>lc_detailed!BJ4/$X$2</f>
-        <v>0.15214611962784025</v>
+        <f>lc_detailed!BK4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F4" s="29">
-        <f>lc_detailed!BK4/$X$2</f>
+        <f>lc_detailed!BL4/$W$2</f>
         <v>0</v>
       </c>
       <c r="G4" s="29">
-        <f>lc_detailed!BL4/$X$2</f>
+        <f>lc_detailed!BM4/$W$2</f>
         <v>0</v>
       </c>
       <c r="H4" s="29">
-        <f>lc_detailed!BM4/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BN4/$W$2</f>
+        <v>0.34050656770373977</v>
       </c>
       <c r="I4" s="29">
-        <f>lc_detailed!BN4/$X$2</f>
-        <v>0.34050656770373977</v>
+        <f>lc_detailed!BO4/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J4" s="29">
-        <f>lc_detailed!BO4/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K4" s="29">
-        <f>lc_detailed!BP4/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ4/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L4" s="29">
-        <f>lc_detailed!BQ4/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR4/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M4" s="29">
-        <f>lc_detailed!BR4/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS4/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N4" s="29">
-        <f>lc_detailed!BS4/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT4/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O4" s="29">
-        <f>lc_detailed!BT4/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!BV4/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P4" s="29">
-        <f>lc_detailed!BV4/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW4/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q4" s="29">
-        <f>lc_detailed!BW4/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R4" s="29">
         <f>lc_detailed!BU4</f>
         <v>-3.14</v>
       </c>
-      <c r="S4" s="29">
+      <c r="R4" s="29">
         <f>lc_detailed!BB4</f>
         <v>115.53269393135753</v>
       </c>
-      <c r="T4" s="29">
+      <c r="S4" s="29">
         <f t="shared" si="0"/>
         <v>2.5336117090209984</v>
       </c>
-      <c r="U4" s="29">
+      <c r="T4" s="29">
         <f t="shared" si="1"/>
         <v>2.5336117090209989</v>
       </c>
+      <c r="U4" s="29"/>
       <c r="V4" s="29"/>
       <c r="W4" s="29"/>
       <c r="X4" s="29"/>
-      <c r="Y4" s="29"/>
-    </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B5" t="str">
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5" t="str">
         <f>lc_detailed!AZ5</f>
         <v>CA_Ethanol_Dehydration_NGfuel</v>
       </c>
+      <c r="B5" s="29">
+        <f>lc_detailed!BH5/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C5" s="29">
-        <f>lc_detailed!BH5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI5/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D5" s="29">
-        <f>lc_detailed!BI5/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ5/$W$2</f>
+        <v>0.14502681211104032</v>
       </c>
       <c r="E5" s="29">
-        <f>lc_detailed!BJ5/$X$2</f>
-        <v>0.14502681211104032</v>
+        <f>lc_detailed!BK5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F5" s="29">
-        <f>lc_detailed!BK5/$X$2</f>
+        <f>lc_detailed!BL5/$W$2</f>
         <v>0</v>
       </c>
       <c r="G5" s="29">
-        <f>lc_detailed!BL5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BM5/$W$2</f>
+        <v>0.41273547391800947</v>
       </c>
       <c r="H5" s="29">
-        <f>lc_detailed!BM5/$X$2</f>
-        <v>0.41273547391800947</v>
+        <f>lc_detailed!BN5/$W$2</f>
+        <v>0.8288013034403614</v>
       </c>
       <c r="I5" s="29">
-        <f>lc_detailed!BN5/$X$2</f>
-        <v>0.8288013034403614</v>
+        <f>lc_detailed!BO5/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J5" s="29">
-        <f>lc_detailed!BO5/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K5" s="29">
-        <f>lc_detailed!BP5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ5/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L5" s="29">
-        <f>lc_detailed!BQ5/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR5/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M5" s="29">
-        <f>lc_detailed!BR5/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS5/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N5" s="29">
-        <f>lc_detailed!BS5/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT5/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O5" s="29">
-        <f>lc_detailed!BT5/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!BV5/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P5" s="29">
-        <f>lc_detailed!BV5/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW5/$W$2</f>
+        <v>-8.4102014092105168</v>
       </c>
       <c r="Q5" s="29">
-        <f>lc_detailed!BW5/$X$2</f>
-        <v>-8.4102014092105168</v>
-      </c>
-      <c r="R5" s="29">
         <f>lc_detailed!BU5</f>
         <v>-3.1399999999999966</v>
       </c>
-      <c r="S5" s="29">
+      <c r="R5" s="29">
         <f>lc_detailed!BB5</f>
         <v>142.25059699693276</v>
       </c>
-      <c r="T5" s="29">
+      <c r="S5" s="29">
         <f t="shared" si="0"/>
         <v>3.119530635897648</v>
       </c>
-      <c r="U5" s="29">
+      <c r="T5" s="29">
         <f t="shared" si="1"/>
         <v>3.1195306358976485</v>
       </c>
+      <c r="U5" s="29"/>
       <c r="V5" s="29"/>
       <c r="W5" s="29"/>
       <c r="X5" s="29"/>
-      <c r="Y5" s="29"/>
-    </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B6" t="str">
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A6" t="str">
         <f>lc_detailed!AZ6</f>
         <v>CA_Ethanol_Dehydration_H2fuel</v>
       </c>
+      <c r="B6" s="29">
+        <f>lc_detailed!BH6/$W$2</f>
+        <v>0.30804920915009643</v>
+      </c>
       <c r="C6" s="29">
-        <f>lc_detailed!BH6/$X$2</f>
-        <v>0.30804920915009643</v>
+        <f>lc_detailed!BI6/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D6" s="29">
-        <f>lc_detailed!BI6/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ6/$W$2</f>
+        <v>0.14502681211104032</v>
       </c>
       <c r="E6" s="29">
-        <f>lc_detailed!BJ6/$X$2</f>
-        <v>0.14502681211104032</v>
+        <f>lc_detailed!BK6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="F6" s="29">
-        <f>lc_detailed!BK6/$X$2</f>
+        <f>lc_detailed!BL6/$W$2</f>
         <v>0</v>
       </c>
       <c r="G6" s="29">
-        <f>lc_detailed!BL6/$X$2</f>
+        <f>lc_detailed!BM6/$W$2</f>
         <v>0</v>
       </c>
       <c r="H6" s="29">
-        <f>lc_detailed!BM6/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BN6/$W$2</f>
+        <v>0.8288013034403614</v>
       </c>
       <c r="I6" s="29">
-        <f>lc_detailed!BN6/$X$2</f>
-        <v>0.8288013034403614</v>
+        <f>lc_detailed!BO6/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J6" s="29">
-        <f>lc_detailed!BO6/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="K6" s="29">
-        <f>lc_detailed!BP6/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BQ6/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L6" s="29">
-        <f>lc_detailed!BQ6/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR6/$W$2</f>
+        <v>1.8656909266504809</v>
       </c>
       <c r="M6" s="29">
-        <f>lc_detailed!BR6/$X$2</f>
-        <v>1.8656909266504809</v>
+        <f>lc_detailed!BS6/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N6" s="29">
-        <f>lc_detailed!BS6/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT6/$W$2</f>
+        <v>7.6055101643215739</v>
       </c>
       <c r="O6" s="29">
-        <f>lc_detailed!BT6/$X$2</f>
-        <v>7.6055101643215739</v>
+        <f>lc_detailed!BV6/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P6" s="29">
-        <f>lc_detailed!BV6/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW6/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q6" s="29">
-        <f>lc_detailed!BW6/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R6" s="29">
         <f>lc_detailed!BU6</f>
         <v>-3.14</v>
       </c>
-      <c r="S6" s="29">
+      <c r="R6" s="29">
         <f>lc_detailed!BB6</f>
         <v>137.4769033235155</v>
       </c>
-      <c r="T6" s="29">
+      <c r="S6" s="29">
         <f t="shared" si="0"/>
         <v>3.0148443711297257</v>
       </c>
-      <c r="U6" s="29">
+      <c r="T6" s="29">
         <f t="shared" si="1"/>
         <v>3.0148443711297261</v>
       </c>
+      <c r="U6" s="29"/>
       <c r="V6" s="29"/>
       <c r="W6" s="29"/>
       <c r="X6" s="29"/>
-      <c r="Y6" s="29"/>
-    </row>
-    <row r="7" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B7" t="str">
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7" t="str">
         <f>lc_detailed!AZ7</f>
         <v>SE_Ethanol_Dehydration_NGfuel_ethanol_biochemical</v>
       </c>
+      <c r="B7" s="29">
+        <f>lc_detailed!BH7/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C7" s="29">
-        <f>lc_detailed!BH7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI7/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D7" s="29">
-        <f>lc_detailed!BI7/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E7" s="29">
-        <f>lc_detailed!BJ7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK7/$W$2</f>
+        <v>-0.65401543344053303</v>
       </c>
       <c r="F7" s="29">
-        <f>lc_detailed!BK7/$X$2</f>
-        <v>-0.65401543344053303</v>
+        <f>lc_detailed!BL7/$W$2</f>
+        <v>11.981390717318295</v>
       </c>
       <c r="G7" s="29">
-        <f>lc_detailed!BL7/$X$2</f>
-        <v>11.981390717318295</v>
+        <f>lc_detailed!BM7/$W$2</f>
+        <v>0.16956915850640997</v>
       </c>
       <c r="H7" s="29">
-        <f>lc_detailed!BM7/$X$2</f>
-        <v>0.16956915850640997</v>
+        <f>lc_detailed!BN7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="I7" s="29">
-        <f>lc_detailed!BN7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO7/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J7" s="29">
-        <f>lc_detailed!BO7/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP7/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K7" s="29">
-        <f>lc_detailed!BP7/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ7/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L7" s="29">
-        <f>lc_detailed!BQ7/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR7/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M7" s="29">
-        <f>lc_detailed!BR7/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS7/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N7" s="29">
-        <f>lc_detailed!BS7/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT7/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O7" s="29">
-        <f>lc_detailed!BT7/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!BV7/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P7" s="29">
-        <f>lc_detailed!BV7/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW7/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q7" s="29">
-        <f>lc_detailed!BW7/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R7" s="29">
         <f>lc_detailed!BU7</f>
         <v>-3.14</v>
       </c>
-      <c r="S7" s="29">
+      <c r="R7" s="29">
         <f>lc_detailed!BB7</f>
         <v>1669.8297288138133</v>
       </c>
-      <c r="T7" s="29">
+      <c r="S7" s="29">
         <f t="shared" si="0"/>
         <v>36.619073000302919</v>
       </c>
-      <c r="U7" s="29">
+      <c r="T7" s="29">
         <f t="shared" si="1"/>
         <v>36.619073000302919</v>
       </c>
+      <c r="U7" s="29"/>
       <c r="V7" s="29"/>
       <c r="W7" s="29"/>
       <c r="X7" s="29"/>
-      <c r="Y7" s="29"/>
-    </row>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B8" t="str">
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8" t="str">
         <f>lc_detailed!AZ8</f>
         <v>SE_Ethanol_Dehydration_H2fuel_ethanol_biochemical</v>
       </c>
+      <c r="B8" s="29">
+        <f>lc_detailed!BH8/$W$2</f>
+        <v>0.30171339336527736</v>
+      </c>
       <c r="C8" s="29">
-        <f>lc_detailed!BH8/$X$2</f>
-        <v>0.30171339336527736</v>
+        <f>lc_detailed!BI8/$W$2</f>
+        <v>0.13417904339355152</v>
       </c>
       <c r="D8" s="29">
-        <f>lc_detailed!BI8/$X$2</f>
-        <v>0.13417904339355152</v>
+        <f>lc_detailed!BJ8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E8" s="29">
-        <f>lc_detailed!BJ8/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK8/$W$2</f>
+        <v>-0.65401543344053303</v>
       </c>
       <c r="F8" s="29">
-        <f>lc_detailed!BK8/$X$2</f>
-        <v>-0.65401543344053303</v>
+        <f>lc_detailed!BL8/$W$2</f>
+        <v>11.981390717318295</v>
       </c>
       <c r="G8" s="29">
-        <f>lc_detailed!BL8/$X$2</f>
-        <v>11.981390717318295</v>
+        <f>lc_detailed!BM8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="H8" s="29">
-        <f>lc_detailed!BM8/$X$2</f>
+        <f>lc_detailed!BN8/$W$2</f>
         <v>0</v>
       </c>
       <c r="I8" s="29">
-        <f>lc_detailed!BN8/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO8/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J8" s="29">
-        <f>lc_detailed!BO8/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP8/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K8" s="29">
-        <f>lc_detailed!BP8/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ8/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L8" s="29">
-        <f>lc_detailed!BQ8/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR8/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M8" s="29">
-        <f>lc_detailed!BR8/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS8/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N8" s="29">
-        <f>lc_detailed!BS8/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT8/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O8" s="29">
-        <f>lc_detailed!BT8/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!BV8/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P8" s="29">
-        <f>lc_detailed!BV8/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW8/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q8" s="29">
-        <f>lc_detailed!BW8/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R8" s="29">
         <f>lc_detailed!BU8</f>
         <v>-3.14</v>
       </c>
-      <c r="S8" s="29">
+      <c r="R8" s="29">
         <f>lc_detailed!BB8</f>
         <v>1675.8555059233772</v>
       </c>
-      <c r="T8" s="29">
+      <c r="S8" s="29">
         <f t="shared" si="0"/>
         <v>36.751217235161782</v>
       </c>
-      <c r="U8" s="29">
+      <c r="T8" s="29">
         <f t="shared" si="1"/>
         <v>36.751217235161789</v>
       </c>
+      <c r="U8" s="29"/>
       <c r="V8" s="29"/>
       <c r="W8" s="29"/>
       <c r="X8" s="29"/>
-      <c r="Y8" s="29"/>
-    </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B9" t="str">
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A9" t="str">
         <f>lc_detailed!AZ9</f>
         <v>CA_Ethanol_Dehydration_NGfuel_ethanol_biochemical</v>
       </c>
+      <c r="B9" s="29">
+        <f>lc_detailed!BH9/$W$2</f>
+        <v>0</v>
+      </c>
       <c r="C9" s="29">
-        <f>lc_detailed!BH9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BI9/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D9" s="29">
-        <f>lc_detailed!BI9/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E9" s="29">
-        <f>lc_detailed!BJ9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK9/$W$2</f>
+        <v>-0.62341237236486724</v>
       </c>
       <c r="F9" s="29">
-        <f>lc_detailed!BK9/$X$2</f>
-        <v>-0.62341237236486724</v>
+        <f>lc_detailed!BL9/$W$2</f>
+        <v>14.614183152615643</v>
       </c>
       <c r="G9" s="29">
-        <f>lc_detailed!BL9/$X$2</f>
-        <v>14.614183152615643</v>
+        <f>lc_detailed!BM9/$W$2</f>
+        <v>0.41273547391800947</v>
       </c>
       <c r="H9" s="29">
-        <f>lc_detailed!BM9/$X$2</f>
-        <v>0.41273547391800947</v>
+        <f>lc_detailed!BN9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="I9" s="29">
-        <f>lc_detailed!BN9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO9/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J9" s="29">
-        <f>lc_detailed!BO9/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP9/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K9" s="29">
-        <f>lc_detailed!BP9/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ9/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L9" s="29">
-        <f>lc_detailed!BQ9/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR9/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M9" s="29">
-        <f>lc_detailed!BR9/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS9/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N9" s="29">
-        <f>lc_detailed!BS9/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT9/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O9" s="29">
-        <f>lc_detailed!BT9/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!BV9/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P9" s="29">
-        <f>lc_detailed!BV9/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW9/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q9" s="29">
-        <f>lc_detailed!BW9/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R9" s="29">
         <f>lc_detailed!BU9</f>
         <v>-3.14</v>
       </c>
-      <c r="S9" s="29">
+      <c r="R9" s="29">
         <f>lc_detailed!BB9</f>
         <v>1802.082644096738</v>
       </c>
-      <c r="T9" s="29">
+      <c r="S9" s="29">
         <f t="shared" si="0"/>
         <v>39.519356230191619</v>
       </c>
-      <c r="U9" s="29">
+      <c r="T9" s="29">
         <f t="shared" si="1"/>
         <v>39.519356230191619</v>
       </c>
+      <c r="U9" s="29"/>
       <c r="V9" s="29"/>
       <c r="W9" s="29"/>
       <c r="X9" s="29"/>
-      <c r="Y9" s="29"/>
-    </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B10" t="str">
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A10" t="str">
         <f>lc_detailed!AZ10</f>
         <v>CA_Ethanol_Dehydration_H2fuel_ethanol_biochemical</v>
       </c>
+      <c r="B10" s="29">
+        <f>lc_detailed!BH10/$W$2</f>
+        <v>0.30804920915009643</v>
+      </c>
       <c r="C10" s="29">
-        <f>lc_detailed!BH10/$X$2</f>
-        <v>0.30804920915009643</v>
+        <f>lc_detailed!BI10/$W$2</f>
+        <v>0.12790046149763876</v>
       </c>
       <c r="D10" s="29">
-        <f>lc_detailed!BI10/$X$2</f>
-        <v>0.12790046149763876</v>
+        <f>lc_detailed!BJ10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="E10" s="29">
-        <f>lc_detailed!BJ10/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BK10/$W$2</f>
+        <v>-0.62341237236486724</v>
       </c>
       <c r="F10" s="29">
-        <f>lc_detailed!BK10/$X$2</f>
-        <v>-0.62341237236486724</v>
+        <f>lc_detailed!BL10/$W$2</f>
+        <v>14.614183152615643</v>
       </c>
       <c r="G10" s="29">
-        <f>lc_detailed!BL10/$X$2</f>
-        <v>14.614183152615643</v>
+        <f>lc_detailed!BM10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="H10" s="29">
-        <f>lc_detailed!BM10/$X$2</f>
+        <f>lc_detailed!BN10/$W$2</f>
         <v>0</v>
       </c>
       <c r="I10" s="29">
-        <f>lc_detailed!BN10/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BO10/$W$2</f>
+        <v>0.25972008040490513</v>
       </c>
       <c r="J10" s="29">
-        <f>lc_detailed!BO10/$X$2</f>
-        <v>0.25972008040490513</v>
+        <f>lc_detailed!BP10/$W$2</f>
+        <v>16.714311159468846</v>
       </c>
       <c r="K10" s="29">
-        <f>lc_detailed!BP10/$X$2</f>
-        <v>16.714311159468846</v>
+        <f>lc_detailed!BQ10/$W$2</f>
+        <v>0.24969769997021227</v>
       </c>
       <c r="L10" s="29">
-        <f>lc_detailed!BQ10/$X$2</f>
-        <v>0.24969769997021227</v>
+        <f>lc_detailed!BR10/$W$2</f>
+        <v>4.9640505619899065</v>
       </c>
       <c r="M10" s="29">
-        <f>lc_detailed!BR10/$X$2</f>
-        <v>4.9640505619899065</v>
+        <f>lc_detailed!BS10/$W$2</f>
+        <v>3.4649122793943513E-2</v>
       </c>
       <c r="N10" s="29">
-        <f>lc_detailed!BS10/$X$2</f>
-        <v>3.4649122793943513E-2</v>
+        <f>lc_detailed!BT10/$W$2</f>
+        <v>11.17572229910791</v>
       </c>
       <c r="O10" s="29">
-        <f>lc_detailed!BT10/$X$2</f>
-        <v>11.17572229910791</v>
+        <f>lc_detailed!BV10/$W$2</f>
+        <v>0</v>
       </c>
       <c r="P10" s="29">
-        <f>lc_detailed!BV10/$X$2</f>
-        <v>0</v>
+        <f>lc_detailed!BW10/$W$2</f>
+        <v>-8.4102014092105257</v>
       </c>
       <c r="Q10" s="29">
-        <f>lc_detailed!BW10/$X$2</f>
-        <v>-8.4102014092105257</v>
-      </c>
-      <c r="R10" s="29">
         <f>lc_detailed!BU10</f>
         <v>-3.14</v>
       </c>
-      <c r="S10" s="29">
+      <c r="R10" s="29">
         <f>lc_detailed!BB10</f>
         <v>1797.3089504233208</v>
       </c>
-      <c r="T10" s="29">
+      <c r="S10" s="29">
         <f t="shared" si="0"/>
         <v>39.414669965423698</v>
       </c>
-      <c r="U10" s="29">
+      <c r="T10" s="29">
         <f t="shared" si="1"/>
         <v>39.414669965423712</v>
       </c>
+      <c r="U10" s="29"/>
       <c r="V10" s="29"/>
       <c r="W10" s="29"/>
       <c r="X10" s="29"/>
-      <c r="Y10" s="29"/>
-    </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B11" s="29"/>
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
       <c r="E11" s="29"/>
@@ -11514,9 +11513,9 @@
       <c r="V11" s="29"/>
       <c r="W11" s="29"/>
       <c r="X11" s="29"/>
-      <c r="Y11" s="29"/>
-    </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B12" s="29"/>
       <c r="C12" s="29"/>
       <c r="D12" s="29"/>
       <c r="E12" s="29"/>
@@ -11539,9 +11538,9 @@
       <c r="V12" s="29"/>
       <c r="W12" s="29"/>
       <c r="X12" s="29"/>
-      <c r="Y12" s="29"/>
-    </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B13" s="29"/>
       <c r="C13" s="29"/>
       <c r="D13" s="29"/>
       <c r="E13" s="29"/>
@@ -11564,9 +11563,9 @@
       <c r="V13" s="29"/>
       <c r="W13" s="29"/>
       <c r="X13" s="29"/>
-      <c r="Y13" s="29"/>
-    </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B14" s="29"/>
       <c r="C14" s="29"/>
       <c r="D14" s="29"/>
       <c r="E14" s="29"/>
@@ -11589,9 +11588,9 @@
       <c r="V14" s="29"/>
       <c r="W14" s="29"/>
       <c r="X14" s="29"/>
-      <c r="Y14" s="29"/>
-    </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B15" s="29"/>
       <c r="C15" s="29"/>
       <c r="D15" s="29"/>
       <c r="E15" s="29"/>
@@ -11614,9 +11613,9 @@
       <c r="V15" s="29"/>
       <c r="W15" s="29"/>
       <c r="X15" s="29"/>
-      <c r="Y15" s="29"/>
-    </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B16" s="29"/>
       <c r="C16" s="29"/>
       <c r="D16" s="29"/>
       <c r="E16" s="29"/>
@@ -11639,9 +11638,9 @@
       <c r="V16" s="29"/>
       <c r="W16" s="29"/>
       <c r="X16" s="29"/>
-      <c r="Y16" s="29"/>
-    </row>
-    <row r="17" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B17" s="29"/>
       <c r="C17" s="29"/>
       <c r="D17" s="29"/>
       <c r="E17" s="29"/>
@@ -11664,9 +11663,9 @@
       <c r="V17" s="29"/>
       <c r="W17" s="29"/>
       <c r="X17" s="29"/>
-      <c r="Y17" s="29"/>
-    </row>
-    <row r="18" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B18" s="29"/>
       <c r="C18" s="29"/>
       <c r="D18" s="29"/>
       <c r="E18" s="29"/>
@@ -11689,9 +11688,9 @@
       <c r="V18" s="29"/>
       <c r="W18" s="29"/>
       <c r="X18" s="29"/>
-      <c r="Y18" s="29"/>
-    </row>
-    <row r="19" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B19" s="29"/>
       <c r="C19" s="29"/>
       <c r="D19" s="29"/>
       <c r="E19" s="29"/>
@@ -11714,9 +11713,9 @@
       <c r="V19" s="29"/>
       <c r="W19" s="29"/>
       <c r="X19" s="29"/>
-      <c r="Y19" s="29"/>
-    </row>
-    <row r="20" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B20" s="29"/>
       <c r="C20" s="29"/>
       <c r="D20" s="29"/>
       <c r="E20" s="29"/>
@@ -11739,9 +11738,9 @@
       <c r="V20" s="29"/>
       <c r="W20" s="29"/>
       <c r="X20" s="29"/>
-      <c r="Y20" s="29"/>
-    </row>
-    <row r="21" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B21" s="29"/>
       <c r="C21" s="29"/>
       <c r="D21" s="29"/>
       <c r="E21" s="29"/>
@@ -11764,9 +11763,9 @@
       <c r="V21" s="29"/>
       <c r="W21" s="29"/>
       <c r="X21" s="29"/>
-      <c r="Y21" s="29"/>
-    </row>
-    <row r="22" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B22" s="29"/>
       <c r="C22" s="29"/>
       <c r="D22" s="29"/>
       <c r="E22" s="29"/>
@@ -11789,9 +11788,9 @@
       <c r="V22" s="29"/>
       <c r="W22" s="29"/>
       <c r="X22" s="29"/>
-      <c r="Y22" s="29"/>
-    </row>
-    <row r="23" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B23" s="29"/>
       <c r="C23" s="29"/>
       <c r="D23" s="29"/>
       <c r="E23" s="29"/>
@@ -11814,9 +11813,9 @@
       <c r="V23" s="29"/>
       <c r="W23" s="29"/>
       <c r="X23" s="29"/>
-      <c r="Y23" s="29"/>
-    </row>
-    <row r="24" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B24" s="29"/>
       <c r="C24" s="29"/>
       <c r="D24" s="29"/>
       <c r="E24" s="29"/>
@@ -11839,9 +11838,9 @@
       <c r="V24" s="29"/>
       <c r="W24" s="29"/>
       <c r="X24" s="29"/>
-      <c r="Y24" s="29"/>
-    </row>
-    <row r="25" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B25" s="29"/>
       <c r="C25" s="29"/>
       <c r="D25" s="29"/>
       <c r="E25" s="29"/>
@@ -11864,9 +11863,9 @@
       <c r="V25" s="29"/>
       <c r="W25" s="29"/>
       <c r="X25" s="29"/>
-      <c r="Y25" s="29"/>
-    </row>
-    <row r="26" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B26" s="29"/>
       <c r="C26" s="29"/>
       <c r="D26" s="29"/>
       <c r="E26" s="29"/>
@@ -11889,9 +11888,9 @@
       <c r="V26" s="29"/>
       <c r="W26" s="29"/>
       <c r="X26" s="29"/>
-      <c r="Y26" s="29"/>
-    </row>
-    <row r="27" spans="3:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B27" s="29"/>
       <c r="C27" s="29"/>
       <c r="D27" s="29"/>
       <c r="E27" s="29"/>
@@ -11914,7 +11913,6 @@
       <c r="V27" s="29"/>
       <c r="W27" s="29"/>
       <c r="X27" s="29"/>
-      <c r="Y27" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>